<commit_message>
feat: add water and building segmentation with distance-to-risk modeling
</commit_message>
<xml_diff>
--- a/drones4health_functions_table.xlsx
+++ b/drones4health_functions_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Category</t>
   </si>
@@ -50,6 +50,15 @@
   </si>
   <si>
     <t>Model localized vector-borne disease transmission risks within a One Health framework, including solid waste micro-accumulation (IMSR), hydric breeding habitat suitability (IRHE), human infection exposure (IRIH), thermal micro-climate stress (IRTS), canopy shelter (IEC), and entomological vulnerability (IEV, IEAD, IFEB).</t>
+  </si>
+  <si>
+    <t>Feature Segmentation &amp; Risk</t>
+  </si>
+  <si>
+    <t>d4h_segment_water(), d4h_segment_buildings(), d4h_distance_to_risk(), d4h_raster_distance()</t>
+  </si>
+  <si>
+    <t>Automate object-based segmentation of water bodies and residential building footprints from ultra-high resolution RGB imagery, compute minimum Euclidean distance matrices, and model vector flight infection exposure tiers.</t>
   </si>
   <si>
     <t>Spatial Grids &amp; Zonation</t>
@@ -428,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -519,6 +528,17 @@
         <v>23</v>
       </c>
     </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>